<commit_message>
feat(test): 盲审 round2 泛词 title 全部移除（React前端/Golang后端）
终审指令：移除『前端工程师/后端工程师』泛词，保留更细划分——
r2_001 前端开发工程师→React前端工程师（双栈取硬性必备 RN）；
r2_002 后端开发工程师→Golang后端工程师（二选一取序首）。
全量校验无泛词 title。重跑评测（归档 1903）：skills F1
0.7487→0.7640；title 失配 11/20，新增强信号——抽取器将
React/Vue 前缀统一泛化为『前端开发工程师』（r2_001/r2_014/r2_015），
入清单供 prompt 迭代
</commit_message>
<xml_diff>
--- a/backend/data/golden_set/review/jd_manual_review_round2.xlsx
+++ b/backend/data/golden_set/review/jd_manual_review_round2.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>前端开发工程师</t>
+          <t>React前端工程师</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>title 与草稿一致；skills 草稿 32→19（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款；双框架（Vue 全家桶 + React Native）无主导方向，保留『前端开发工程师』（终审细化口径下不可单一框架前缀，否则失真）</t>
+          <t>title 按终审口径细分（移除泛词『前端开发工程师』）：双栈（RN+Vue+小程序+原生）取硬性必备 React Native（『无原生+RN 开发经验者不考虑』），格式对齐 r2_014『React前端工程师』；skills 19 项（DOM/BOM/AJAX 等 JS 子能力不单列，对齐 round1 粒度）；无学历/年限条款</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>后端开发工程师</t>
+          <t>Golang后端工程师</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>草稿 skills 9→8（AI 工具属『附加项』移 bonus）；数据结构与算法为通用基础不单列；3-5 年经验；语言为 Golang 或 Python 二选一、无主导语言，保留『后端开发工程师』（终审细化口径下不可单语言前缀，否则失真）</t>
+          <t>title 按终审口径细分（移除泛词『后端开发工程师』）：『熟练掌握 Golang 或 Python』二选一取序首 Golang，格式对齐 r2_019『Java后端工程师』；skills 8 项（AI 工具属『附加项』移 bonus；数据结构与算法为通用基础不单列）；3-5 年经验</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">

</xml_diff>